<commit_message>
templates: eleven more built in (cover letter, memo, meeting agenda and project proposal; expense report, stock list, weekly planner and grade book; quarterly review, lesson and portfolio), each drawn in the gallery and in every language; the gallery's files and pictures made again by today's engines
</commit_message>
<xml_diff>
--- a/packages/templates/files/sheet-invoice.xlsx
+++ b/packages/templates/files/sheet-invoice.xlsx
@@ -395,7 +395,7 @@
       </c>
       <c r="D3" s="6">
         <f>TODAY()</f>
-        <v>46308</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="4">
@@ -411,7 +411,7 @@
       </c>
       <c r="D4" s="6">
         <f>D3+30</f>
-        <v>46338</v>
+        <v>46345</v>
       </c>
     </row>
     <row r="6">

</xml_diff>